<commit_message>
Coleta automática em 16-12-2025 20:16
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5082,7 +5082,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5152,7 +5152,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5432,7 +5432,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5502,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 17-12-2025 20:16
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5082,7 +5082,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5152,7 +5152,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5432,7 +5432,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5502,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 19-12-2025 20:16
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5082,7 +5082,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5152,7 +5152,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5432,7 +5432,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5502,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 24-12-2025 20:16
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5082,7 +5082,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5152,7 +5152,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5432,7 +5432,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5502,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 25-12-2025 20:16
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5082,7 +5082,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5152,7 +5152,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5432,7 +5432,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5502,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 26-12-2025 20:15
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5082,7 +5082,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5152,7 +5152,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5432,7 +5432,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5502,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 28-12-2025 20:17
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5082,7 +5082,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5152,7 +5152,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5432,7 +5432,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5502,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 02-01-2026 20:16
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5082,7 +5082,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5152,7 +5152,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5432,7 +5432,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5502,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 05-01-2026 20:17
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_Limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_Limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5082,7 +5082,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5152,7 +5152,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5432,7 +5432,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5502,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>